<commit_message>
Add public Zoom links/IDs to Miami and Orlando club sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WnemgMevyHw3X6dXZcvQwV
</commit_message>
<xml_diff>
--- a/docs/Miami-Toastmasters-Clubs.xlsx
+++ b/docs/Miami-Toastmasters-Clubs.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Weekly Schedule'!$A$1:$P$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Weekly Schedule'!$A$1:$T$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P68"/>
+  <dimension ref="A1:T68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -524,6 +524,10 @@
     <col width="34" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="36" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -607,6 +611,26 @@
           <t>Day/time as listed</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Zoom link</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Zoom meeting ID</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Zoom passcode</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>How to get in online</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -681,6 +705,22 @@
           <t>2nd and 4th Monday (except holidays) · 12:00 pm - 1:00 pm</t>
         </is>
       </c>
+      <c r="Q2" s="5" t="inlineStr"/>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>380 489 6491</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>Grove2026</t>
+        </is>
+      </c>
+      <c r="T2" s="6" t="inlineStr">
+        <is>
+          <t>Posted in club website</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -755,6 +795,14 @@
           <t>1st and 3rd Monday · 12:00 PM - 1:00 PM</t>
         </is>
       </c>
+      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="5" t="inlineStr"/>
+      <c r="S3" s="5" t="inlineStr"/>
+      <c r="T3" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -829,6 +877,14 @@
           <t>Monday · 5:30 PM</t>
         </is>
       </c>
+      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="R4" s="5" t="inlineStr"/>
+      <c r="S4" s="5" t="inlineStr"/>
+      <c r="T4" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -903,6 +959,14 @@
           <t>Monday (1st, 2nd, and Third Monday Only) · 6:30 PM ( No Meetings on Holidays)</t>
         </is>
       </c>
+      <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" s="5" t="inlineStr"/>
+      <c r="T5" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -977,6 +1041,14 @@
           <t>Monday Evenings · 6:30 pm - 7:30 pm</t>
         </is>
       </c>
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr"/>
+      <c r="S6" s="5" t="inlineStr"/>
+      <c r="T6" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1051,6 +1123,14 @@
           <t>Mondays · 6:45 pm - 8:20pm</t>
         </is>
       </c>
+      <c r="Q7" s="5" t="inlineStr"/>
+      <c r="R7" s="5" t="inlineStr"/>
+      <c r="S7" s="5" t="inlineStr"/>
+      <c r="T7" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1125,6 +1205,26 @@
           <t>1st Monday · 7.00pm-9.00pm</t>
         </is>
       </c>
+      <c r="Q8" s="7" t="inlineStr">
+        <is>
+          <t>https://us02web.zoom.us/j/85744117242?pwd=aExTRDFuL2RPRHpjbUtYUHpZRldvUT09</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>857 4411 7242</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>welcome</t>
+        </is>
+      </c>
+      <c r="T8" s="6" t="inlineStr">
+        <is>
+          <t>Posted in club website</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1197,6 +1297,14 @@
       <c r="P9" s="6" t="inlineStr">
         <is>
           <t>Monday · 7:15 pm - 8:45 pm</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr"/>
+      <c r="S9" s="5" t="inlineStr"/>
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
         </is>
       </c>
     </row>
@@ -1269,6 +1377,14 @@
           <t>Monday · 7:30 pm - 9:15 pm</t>
         </is>
       </c>
+      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr"/>
+      <c r="S10" s="5" t="inlineStr"/>
+      <c r="T10" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -1343,6 +1459,14 @@
           <t>Tuesdays · 12:05 - 12:55PM ET</t>
         </is>
       </c>
+      <c r="Q11" s="12" t="inlineStr"/>
+      <c r="R11" s="12" t="inlineStr"/>
+      <c r="S11" s="12" t="inlineStr"/>
+      <c r="T11" s="13" t="inlineStr">
+        <is>
+          <t>Club site says meetings are on Zoom; request link from club</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -1417,6 +1541,14 @@
           <t>Tuesday and Thursday · Tue 6:30 - 7:30 PM | Thu 7:30 - 8:30 AM</t>
         </is>
       </c>
+      <c r="Q12" s="12" t="inlineStr"/>
+      <c r="R12" s="12" t="inlineStr"/>
+      <c r="S12" s="12" t="inlineStr"/>
+      <c r="T12" s="13" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1487,6 +1619,14 @@
           <t>2 nd &amp; 4th  Tuesday · 6:30 pm</t>
         </is>
       </c>
+      <c r="Q13" s="12" t="inlineStr"/>
+      <c r="R13" s="12" t="inlineStr"/>
+      <c r="S13" s="12" t="inlineStr"/>
+      <c r="T13" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -1561,6 +1701,14 @@
           <t>Tuesdays on Zoom · 6:30 p.m. - 7:45 p.m.</t>
         </is>
       </c>
+      <c r="Q14" s="12" t="inlineStr"/>
+      <c r="R14" s="12" t="inlineStr"/>
+      <c r="S14" s="12" t="inlineStr"/>
+      <c r="T14" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -1635,6 +1783,14 @@
           <t>1st &amp; 3rd Tuesday · 6:30 p.m.</t>
         </is>
       </c>
+      <c r="Q15" s="12" t="inlineStr"/>
+      <c r="R15" s="12" t="inlineStr"/>
+      <c r="S15" s="12" t="inlineStr"/>
+      <c r="T15" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -1709,6 +1865,14 @@
           <t>Tuesday · 6:30 pm - 8:30 pm</t>
         </is>
       </c>
+      <c r="Q16" s="12" t="inlineStr"/>
+      <c r="R16" s="12" t="inlineStr"/>
+      <c r="S16" s="12" t="inlineStr"/>
+      <c r="T16" s="13" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -1783,6 +1947,14 @@
           <t>1st &amp; 3rd Tuesday · 7:00 pm - 8:30 pm</t>
         </is>
       </c>
+      <c r="Q17" s="12" t="inlineStr"/>
+      <c r="R17" s="12" t="inlineStr"/>
+      <c r="S17" s="12" t="inlineStr"/>
+      <c r="T17" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -1857,6 +2029,26 @@
           <t>2nd &amp; 4th Tuesday · 7:00 pm</t>
         </is>
       </c>
+      <c r="Q18" s="14" t="inlineStr">
+        <is>
+          <t>https://zoom.us/j/98574620252?pwd=A4sRvpkypAEOBGpUznWW2pyKeT5wdM.1</t>
+        </is>
+      </c>
+      <c r="R18" s="12" t="inlineStr">
+        <is>
+          <t>985 7462 0252</t>
+        </is>
+      </c>
+      <c r="S18" s="12" t="inlineStr">
+        <is>
+          <t>137427</t>
+        </is>
+      </c>
+      <c r="T18" s="13" t="inlineStr">
+        <is>
+          <t>Posted in toastmasters directory</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1931,6 +2123,14 @@
           <t>2nd &amp; 4th Tuesdays (see website) · 07:05 PM</t>
         </is>
       </c>
+      <c r="Q19" s="12" t="inlineStr"/>
+      <c r="R19" s="12" t="inlineStr"/>
+      <c r="S19" s="12" t="inlineStr"/>
+      <c r="T19" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -2005,6 +2205,22 @@
           <t>Tuesday · 7:30 pm</t>
         </is>
       </c>
+      <c r="Q20" s="14" t="inlineStr">
+        <is>
+          <t>https://us02web.zoom.us/j/83511038849</t>
+        </is>
+      </c>
+      <c r="R20" s="12" t="inlineStr">
+        <is>
+          <t>835 1103 8849</t>
+        </is>
+      </c>
+      <c r="S20" s="12" t="inlineStr"/>
+      <c r="T20" s="13" t="inlineStr">
+        <is>
+          <t>Posted on club website (link written with spaces there)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2079,6 +2295,14 @@
           <t>Wednesday · 7:30 am - 8:30 am</t>
         </is>
       </c>
+      <c r="Q21" s="5" t="inlineStr"/>
+      <c r="R21" s="5" t="inlineStr"/>
+      <c r="S21" s="5" t="inlineStr"/>
+      <c r="T21" s="6" t="inlineStr">
+        <is>
+          <t>Club site says meetings are on Zoom; request link from club</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2157,6 +2381,14 @@
           <t>Wednesday · 7:45 am - 8:45 am</t>
         </is>
       </c>
+      <c r="Q22" s="5" t="inlineStr"/>
+      <c r="R22" s="5" t="inlineStr"/>
+      <c r="S22" s="5" t="inlineStr"/>
+      <c r="T22" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2235,6 +2467,14 @@
           <t>3rd Wednesdays · 10:00 AM</t>
         </is>
       </c>
+      <c r="Q23" s="5" t="inlineStr"/>
+      <c r="R23" s="5" t="inlineStr"/>
+      <c r="S23" s="5" t="inlineStr"/>
+      <c r="T23" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2309,6 +2549,14 @@
           <t>Every 2nd And 4th Wednesdays · 12:00 pm -1:00 pm EDT</t>
         </is>
       </c>
+      <c r="Q24" s="5" t="inlineStr"/>
+      <c r="R24" s="5" t="inlineStr"/>
+      <c r="S24" s="5" t="inlineStr"/>
+      <c r="T24" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2383,6 +2631,14 @@
           <t>2nd &amp; 4th Wednesday · 12:00 pm</t>
         </is>
       </c>
+      <c r="Q25" s="5" t="inlineStr"/>
+      <c r="R25" s="5" t="inlineStr"/>
+      <c r="S25" s="5" t="inlineStr"/>
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2457,6 +2713,18 @@
           <t>1st and 3rd WEDNESDAY (ONLINE) · 12PM-1PM</t>
         </is>
       </c>
+      <c r="Q26" s="7" t="inlineStr">
+        <is>
+          <t>https://us02web.zoom.us/j/84490264148</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr"/>
+      <c r="S26" s="5" t="inlineStr"/>
+      <c r="T26" s="6" t="inlineStr">
+        <is>
+          <t>Posted in toastmasters directory</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2531,6 +2799,14 @@
           <t>Second &amp; Fourth Wednesday · 12:00 pm - 1:00 pm</t>
         </is>
       </c>
+      <c r="Q27" s="5" t="inlineStr"/>
+      <c r="R27" s="5" t="inlineStr"/>
+      <c r="S27" s="5" t="inlineStr"/>
+      <c r="T27" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2605,6 +2881,14 @@
           <t>Last Wednesday · 12:00 PM</t>
         </is>
       </c>
+      <c r="Q28" s="5" t="inlineStr"/>
+      <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" s="5" t="inlineStr"/>
+      <c r="T28" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2683,6 +2967,14 @@
           <t>1st &amp; 3rd Wednesdays · 12:00 PM</t>
         </is>
       </c>
+      <c r="Q29" s="5" t="inlineStr"/>
+      <c r="R29" s="5" t="inlineStr"/>
+      <c r="S29" s="5" t="inlineStr"/>
+      <c r="T29" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2761,6 +3053,14 @@
           <t>Wednesday · 12:00 pm</t>
         </is>
       </c>
+      <c r="Q30" s="5" t="inlineStr"/>
+      <c r="R30" s="5" t="inlineStr"/>
+      <c r="S30" s="5" t="inlineStr"/>
+      <c r="T30" s="6" t="inlineStr">
+        <is>
+          <t>Club site says meetings are on Zoom; request link from club</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2835,6 +3135,14 @@
           <t>1st Wednesday · 12:00 - 1:30 PM</t>
         </is>
       </c>
+      <c r="Q31" s="5" t="inlineStr"/>
+      <c r="R31" s="5" t="inlineStr"/>
+      <c r="S31" s="5" t="inlineStr"/>
+      <c r="T31" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2909,6 +3217,14 @@
           <t>Every Other Wednesday (Employees Only) · 12:00 - 1:00 PM</t>
         </is>
       </c>
+      <c r="Q32" s="5" t="inlineStr"/>
+      <c r="R32" s="5" t="inlineStr"/>
+      <c r="S32" s="5" t="inlineStr"/>
+      <c r="T32" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2983,6 +3299,14 @@
           <t>Every other Wednesday · 12:00 p.m.</t>
         </is>
       </c>
+      <c r="Q33" s="5" t="inlineStr"/>
+      <c r="R33" s="5" t="inlineStr"/>
+      <c r="S33" s="5" t="inlineStr"/>
+      <c r="T33" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3057,6 +3381,14 @@
           <t>Wednesdays · 12:00</t>
         </is>
       </c>
+      <c r="Q34" s="5" t="inlineStr"/>
+      <c r="R34" s="5" t="inlineStr"/>
+      <c r="S34" s="5" t="inlineStr"/>
+      <c r="T34" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3131,6 +3463,14 @@
           <t>2nd &amp; 4th Wednesdays · 12:00 PM</t>
         </is>
       </c>
+      <c r="Q35" s="5" t="inlineStr"/>
+      <c r="R35" s="5" t="inlineStr"/>
+      <c r="S35" s="5" t="inlineStr"/>
+      <c r="T35" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3201,6 +3541,14 @@
           <t>Wednesday · 1:00 pm</t>
         </is>
       </c>
+      <c r="Q36" s="5" t="inlineStr"/>
+      <c r="R36" s="5" t="inlineStr"/>
+      <c r="S36" s="5" t="inlineStr"/>
+      <c r="T36" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3275,6 +3623,14 @@
           <t>1st Wednesday · 2:30 PM</t>
         </is>
       </c>
+      <c r="Q37" s="5" t="inlineStr"/>
+      <c r="R37" s="5" t="inlineStr"/>
+      <c r="S37" s="5" t="inlineStr"/>
+      <c r="T37" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3349,6 +3705,14 @@
           <t>Wednesdays · 4:00 PM Eastern</t>
         </is>
       </c>
+      <c r="Q38" s="5" t="inlineStr"/>
+      <c r="R38" s="5" t="inlineStr"/>
+      <c r="S38" s="5" t="inlineStr"/>
+      <c r="T38" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3423,6 +3787,14 @@
           <t>2nd &amp; 4th Wednesday · 6:30pm</t>
         </is>
       </c>
+      <c r="Q39" s="5" t="inlineStr"/>
+      <c r="R39" s="5" t="inlineStr"/>
+      <c r="S39" s="5" t="inlineStr"/>
+      <c r="T39" s="6" t="inlineStr">
+        <is>
+          <t>Club site says meetings are on Zoom; request link from club</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3497,6 +3869,14 @@
           <t>Wednesday · 6:30 PM</t>
         </is>
       </c>
+      <c r="Q40" s="5" t="inlineStr"/>
+      <c r="R40" s="5" t="inlineStr"/>
+      <c r="S40" s="5" t="inlineStr"/>
+      <c r="T40" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3571,6 +3951,14 @@
           <t>2nd &amp; 4th Wednesday of every month · 6:45 p.m.</t>
         </is>
       </c>
+      <c r="Q41" s="5" t="inlineStr"/>
+      <c r="R41" s="5" t="inlineStr"/>
+      <c r="S41" s="5" t="inlineStr"/>
+      <c r="T41" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3645,6 +4033,14 @@
           <t>2nd &amp; 4th Wednesday · 6:45 pm</t>
         </is>
       </c>
+      <c r="Q42" s="5" t="inlineStr"/>
+      <c r="R42" s="5" t="inlineStr"/>
+      <c r="S42" s="5" t="inlineStr"/>
+      <c r="T42" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3719,6 +4115,14 @@
           <t>Every Wednesday · 7:00 PM - 8:30 PM</t>
         </is>
       </c>
+      <c r="Q43" s="5" t="inlineStr"/>
+      <c r="R43" s="5" t="inlineStr"/>
+      <c r="S43" s="5" t="inlineStr"/>
+      <c r="T43" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3793,6 +4197,14 @@
           <t>2nd &amp; 4th Wednesday · 7:00 pm</t>
         </is>
       </c>
+      <c r="Q44" s="5" t="inlineStr"/>
+      <c r="R44" s="5" t="inlineStr"/>
+      <c r="S44" s="5" t="inlineStr"/>
+      <c r="T44" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3867,6 +4279,22 @@
           <t>Wednesday · 7:00 PM</t>
         </is>
       </c>
+      <c r="Q45" s="5" t="inlineStr"/>
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>781 9452 4853</t>
+        </is>
+      </c>
+      <c r="S45" s="5" t="inlineStr">
+        <is>
+          <t>tolo9400</t>
+        </is>
+      </c>
+      <c r="T45" s="6" t="inlineStr">
+        <is>
+          <t>Posted in toastmasters directory</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3941,6 +4369,14 @@
           <t>Wednesday · 7:00 pm</t>
         </is>
       </c>
+      <c r="Q46" s="5" t="inlineStr"/>
+      <c r="R46" s="5" t="inlineStr"/>
+      <c r="S46" s="5" t="inlineStr"/>
+      <c r="T46" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4015,6 +4451,18 @@
           <t>Wednesday · 7:30 pm - 8:30 pm (EST)</t>
         </is>
       </c>
+      <c r="Q47" s="7" t="inlineStr">
+        <is>
+          <t>https://us02web.zoom.us/j/6973415645?pwd=Qm9vOWNkZWR3R0JCc1NJY2EwZnowUT09</t>
+        </is>
+      </c>
+      <c r="R47" s="5" t="inlineStr"/>
+      <c r="S47" s="5" t="inlineStr"/>
+      <c r="T47" s="6" t="inlineStr">
+        <is>
+          <t>Posted in toastmasters directory</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
@@ -4089,6 +4537,18 @@
           <t>Thursday · 7:00 am</t>
         </is>
       </c>
+      <c r="Q48" s="14" t="inlineStr">
+        <is>
+          <t>https://zoom.us/j/451259286</t>
+        </is>
+      </c>
+      <c r="R48" s="12" t="inlineStr"/>
+      <c r="S48" s="12" t="inlineStr"/>
+      <c r="T48" s="13" t="inlineStr">
+        <is>
+          <t>Posted in toastmasters directory</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
@@ -4163,6 +4623,14 @@
           <t>Thursdays · 7:30am to 8:45am</t>
         </is>
       </c>
+      <c r="Q49" s="12" t="inlineStr"/>
+      <c r="R49" s="12" t="inlineStr"/>
+      <c r="S49" s="12" t="inlineStr"/>
+      <c r="T49" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
@@ -4237,6 +4705,14 @@
           <t>Thursday · 12:00 - 1:30 pm</t>
         </is>
       </c>
+      <c r="Q50" s="12" t="inlineStr"/>
+      <c r="R50" s="12" t="inlineStr"/>
+      <c r="S50" s="12" t="inlineStr"/>
+      <c r="T50" s="13" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
@@ -4311,6 +4787,14 @@
           <t>Every Thursday · 12:00 pm</t>
         </is>
       </c>
+      <c r="Q51" s="12" t="inlineStr"/>
+      <c r="R51" s="12" t="inlineStr"/>
+      <c r="S51" s="12" t="inlineStr"/>
+      <c r="T51" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
@@ -4385,6 +4869,14 @@
           <t>THURSDAY EXCEPT FOR 2ND THUR OF MONTH · 12:30 pm</t>
         </is>
       </c>
+      <c r="Q52" s="12" t="inlineStr"/>
+      <c r="R52" s="12" t="inlineStr"/>
+      <c r="S52" s="12" t="inlineStr"/>
+      <c r="T52" s="13" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
@@ -4459,6 +4951,14 @@
           <t>Thursdays · 4:00 PM</t>
         </is>
       </c>
+      <c r="Q53" s="12" t="inlineStr"/>
+      <c r="R53" s="12" t="inlineStr"/>
+      <c r="S53" s="12" t="inlineStr"/>
+      <c r="T53" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
@@ -4533,6 +5033,14 @@
           <t>First and Third Thursdays · 4:15 pm-5:15 pm</t>
         </is>
       </c>
+      <c r="Q54" s="12" t="inlineStr"/>
+      <c r="R54" s="12" t="inlineStr"/>
+      <c r="S54" s="12" t="inlineStr"/>
+      <c r="T54" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
@@ -4607,6 +5115,14 @@
           <t>Thursdays · 6:00 pm</t>
         </is>
       </c>
+      <c r="Q55" s="12" t="inlineStr"/>
+      <c r="R55" s="12" t="inlineStr"/>
+      <c r="S55" s="12" t="inlineStr"/>
+      <c r="T55" s="13" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
@@ -4681,6 +5197,14 @@
           <t>Every Thursday · 6:15 pm - 7:30 pm</t>
         </is>
       </c>
+      <c r="Q56" s="12" t="inlineStr"/>
+      <c r="R56" s="12" t="inlineStr"/>
+      <c r="S56" s="12" t="inlineStr"/>
+      <c r="T56" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
@@ -4751,6 +5275,14 @@
           <t>2nd &amp; 4th Thursday · 6:30 p.m. - 8:00 p.m.</t>
         </is>
       </c>
+      <c r="Q57" s="12" t="inlineStr"/>
+      <c r="R57" s="12" t="inlineStr"/>
+      <c r="S57" s="12" t="inlineStr"/>
+      <c r="T57" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
@@ -4825,6 +5357,14 @@
           <t>Thursday · 6:30 pm - 7:30 pm</t>
         </is>
       </c>
+      <c r="Q58" s="12" t="inlineStr"/>
+      <c r="R58" s="12" t="inlineStr"/>
+      <c r="S58" s="12" t="inlineStr"/>
+      <c r="T58" s="13" t="inlineStr">
+        <is>
+          <t>Club site says meetings are on Zoom; request link from club</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
@@ -4903,6 +5443,18 @@
           <t>3rd THURSDAY · 7:00 pm (EST)</t>
         </is>
       </c>
+      <c r="Q59" s="12" t="inlineStr"/>
+      <c r="R59" s="12" t="inlineStr">
+        <is>
+          <t>821 3347 6040</t>
+        </is>
+      </c>
+      <c r="S59" s="12" t="inlineStr"/>
+      <c r="T59" s="13" t="inlineStr">
+        <is>
+          <t>Posted in toastmasters directory</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
@@ -4977,6 +5529,14 @@
           <t>1st &amp; 3rd Thursday · 7:15 pm</t>
         </is>
       </c>
+      <c r="Q60" s="12" t="inlineStr"/>
+      <c r="R60" s="12" t="inlineStr"/>
+      <c r="S60" s="12" t="inlineStr"/>
+      <c r="T60" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5051,6 +5611,14 @@
           <t>Friday · 7:15 am - 8:30 am (starts promptly)</t>
         </is>
       </c>
+      <c r="Q61" s="5" t="inlineStr"/>
+      <c r="R61" s="5" t="inlineStr"/>
+      <c r="S61" s="5" t="inlineStr"/>
+      <c r="T61" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5129,6 +5697,14 @@
           <t>Fridays · 5:30 PM - 6:30 PM</t>
         </is>
       </c>
+      <c r="Q62" s="5" t="inlineStr"/>
+      <c r="R62" s="5" t="inlineStr"/>
+      <c r="S62" s="5" t="inlineStr"/>
+      <c r="T62" s="6" t="inlineStr">
+        <is>
+          <t>In person only</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
@@ -5203,6 +5779,14 @@
           <t>Saturday · 8:00 AM (Miami/Eastern Time)</t>
         </is>
       </c>
+      <c r="Q63" s="12" t="inlineStr"/>
+      <c r="R63" s="12" t="inlineStr"/>
+      <c r="S63" s="12" t="inlineStr"/>
+      <c r="T63" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
@@ -5277,6 +5861,14 @@
           <t>Saturday · 9 AM - 10:45 AM</t>
         </is>
       </c>
+      <c r="Q64" s="12" t="inlineStr"/>
+      <c r="R64" s="12" t="inlineStr"/>
+      <c r="S64" s="12" t="inlineStr"/>
+      <c r="T64" s="13" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
@@ -5355,6 +5947,14 @@
           <t>2nd &amp; 4th Saturday · 10:00 AM (Miami/Eastern Time)</t>
         </is>
       </c>
+      <c r="Q65" s="12" t="inlineStr"/>
+      <c r="R65" s="12" t="inlineStr"/>
+      <c r="S65" s="12" t="inlineStr"/>
+      <c r="T65" s="13" t="inlineStr">
+        <is>
+          <t>Club site says meetings are on Zoom; request link from club</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
@@ -5429,6 +6029,14 @@
           <t>Saturdays · 11:00 A.M.</t>
         </is>
       </c>
+      <c r="Q66" s="12" t="inlineStr"/>
+      <c r="R66" s="12" t="inlineStr"/>
+      <c r="S66" s="12" t="inlineStr"/>
+      <c r="T66" s="13" t="inlineStr">
+        <is>
+          <t>Club site says meetings are on Zoom; request link from club</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5493,6 +6101,14 @@
         <v>17.7</v>
       </c>
       <c r="P67" s="6" t="inlineStr"/>
+      <c r="Q67" s="5" t="inlineStr"/>
+      <c r="R67" s="5" t="inlineStr"/>
+      <c r="S67" s="5" t="inlineStr"/>
+      <c r="T67" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5557,9 +6173,17 @@
         <v>20.9</v>
       </c>
       <c r="P68" s="6" t="inlineStr"/>
+      <c r="Q68" s="5" t="inlineStr"/>
+      <c r="R68" s="5" t="inlineStr"/>
+      <c r="S68" s="5" t="inlineStr"/>
+      <c r="T68" s="6" t="inlineStr">
+        <is>
+          <t>Ask the club for the link (email in this row)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P68"/>
+  <autoFilter ref="A1:T68"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
@@ -5574,112 +6198,118 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N64" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N58" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N60" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N61" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N62" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N63" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N64" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N65" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N66" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N67" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N68" r:id="rId125"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5691,7 +6321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -5728,26 +6358,33 @@
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>"How often": monthly clubs such as "2nd &amp; 4th Tuesday of month" meet only in those weeks. The last column shows the day/time exactly as the club lists it.</t>
+          <t>Zoom columns: filled only when the club posts its link publicly (in the Toastmasters directory or on its own website). Most clubs email the link to guests instead.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>"Membership may be restricted" usually means a company or government club. Guests are often welcome, but call first.</t>
+          <t>"How often": monthly clubs such as "2nd &amp; 4th Tuesday of month" meet only in those weeks. The last column shows the day/time exactly as the club lists it.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>Contact email and phone are the ones each club publishes in the Toastmasters directory; they can go stale, so confirm before driving over.</t>
+          <t>"Membership may be restricted" usually means a company or government club. Guests are often welcome, but call first.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Contact email and phone are the ones each club publishes in the Toastmasters directory; they can go stale, so confirm before driving over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Miles = straight-line distance from downtown Miami.</t>
         </is>

</xml_diff>